<commit_message>
Make the results downloadable: one-click ZIP bundle, download band, print-ready workbook
- NW_Site_Network_Pack.zip bundles the KMZ, the Excel report, KML, CSV and README
- download page gets a prominent Download both / map / report band at the top
- every workbook sheet is set up for print/PDF export with headers, footers and page numbers

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/network/NW_Network_Site_Database.xlsx
+++ b/network/NW_Network_Site_Database.xlsx
@@ -19,8 +19,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sites'!$A$4:$P$110</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Sites'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'High Sites'!$A$4:$N$24</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'High Sites'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Towns'!$A$4:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Quality'!$A$4:$F$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Data Quality'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Source (as captured)'!$A$4:$H$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1432,7 +1434,7 @@
   <sheetPr>
     <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1882,7 +1884,16 @@
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="A40:B40"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FOverview</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -8892,8 +8903,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P109" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P110" r:id="rId106"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FSites</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -10133,8 +10152,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId20"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FHigh Sites</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -10143,7 +10170,7 @@
   <sheetPr>
     <tabColor rgb="0070AD47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -10790,7 +10817,16 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FTowns</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -10800,7 +10836,7 @@
   <sheetPr>
     <tabColor rgb="00ED7D31"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -11254,7 +11290,16 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FRemote links</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -11263,7 +11308,7 @@
   <sheetPr>
     <tabColor rgb="00C00000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -12288,7 +12333,16 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FData quality</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -12297,7 +12351,7 @@
   <sheetPr>
     <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -15930,6 +15984,15 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K6F6F6FNorth West site network - Current Technology&amp;R&amp;8 &amp;K6F6F6FSource rows</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K6F6F6FBuilt from the CURRENT TECHNOLOGY sheet, rows 40-145&amp;R&amp;8 &amp;K6F6F6FPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>